<commit_message>
Fix DCF pipeline, PEG ratio, chart generation and project workflow
</commit_message>
<xml_diff>
--- a/report/Final_Report.xlsx
+++ b/report/Final_Report.xlsx
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1884.8</v>
+        <v>1851.5</v>
       </c>
     </row>
     <row r="6">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>1024.14</v>
+        <v>436.01</v>
       </c>
     </row>
     <row r="7">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>26.07</v>
+        <v>25.58</v>
       </c>
     </row>
     <row r="9">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>3.82</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="10">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1884.800048828125</v>
+        <v>1851.5</v>
       </c>
     </row>
     <row r="17">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>1973.319473145414</v>
+        <v>1974.002546119542</v>
       </c>
     </row>
     <row r="18">
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>2003.060986647091</v>
+        <v>2003.733254335848</v>
       </c>
     </row>
     <row r="19">
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>2032.802500148768</v>
+        <v>2033.463962552154</v>
       </c>
     </row>
     <row r="20"/>
@@ -777,12 +777,12 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>1024.14</t>
+          <t>436.01</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>1884.8</t>
+          <t>1851.5</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>1884.8</t>
+          <t>1851.5</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>26.07</t>
+          <t>25.58</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>3.82</t>
+          <t>3.76</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>59.85</t>
+          <t>53.85</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">

</xml_diff>